<commit_message>
Updated ESP model - 2025-09-13 09:17
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ESP/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ESP\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C2A078E-47F9-44C9-926B-F6EDFE41976B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F28BC14F-EA47-43D9-9328-5A768A673252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7626,7 +7626,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E245BE3D-6058-4576-97CD-F19635DB0152}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D047537-3E05-45B4-8EAF-D52E70C3ACC8}">
   <dimension ref="B9:N58"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9506,7 +9506,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FF14526-F5B8-432E-8B35-35B750709645}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2434490-698A-43CD-8975-0670D47B1251}">
   <dimension ref="B9:AB156"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20084,7 +20084,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F813168-9FAC-46A2-90D4-00FCDD5454FE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EDB2BB2-CBDF-4AD5-B33E-27854AD6A06B}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ESP model - 2025-09-13 09:59
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ESP/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ESP\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F28BC14F-EA47-43D9-9328-5A768A673252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6261961-5D39-4966-B650-2F788305A7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7626,7 +7626,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D047537-3E05-45B4-8EAF-D52E70C3ACC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{840FFA64-CBCA-42FA-98CC-3F9914C451D4}">
   <dimension ref="B9:N58"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9506,7 +9506,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2434490-698A-43CD-8975-0670D47B1251}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEDD7DCF-6EC3-4080-886A-E5CF5B1CB974}">
   <dimension ref="B9:AB156"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20084,7 +20084,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EDB2BB2-CBDF-4AD5-B33E-27854AD6A06B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1AB6527-F0BC-463D-B1A6-9E7C5DF78235}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>